<commit_message>
add temp inputs. add input cap fft
</commit_message>
<xml_diff>
--- a/data/capacitor_data.xlsx
+++ b/data/capacitor_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://renesasgroup-my.sharepoint.com/personal/gary_kidwell_wz_renesas_com/Documents/python/charger/mathmodels/3lvlbuck/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://renesasgroup-my.sharepoint.com/personal/gary_kidwell_wz_renesas_com/Documents/python/charger/mathmodels/pdis_2or3lvl_bb/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="200" documentId="8_{991A3E6A-3540-42E7-8DD1-010EE75D978B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12D674BF-2253-4BF9-A84B-7F564776BA3F}"/>
+  <xr:revisionPtr revIDLastSave="219" documentId="8_{991A3E6A-3540-42E7-8DD1-010EE75D978B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42804F92-AF31-43B4-889B-E6ECC3F8B765}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="15" windowWidth="15330" windowHeight="10485" xr2:uid="{08943A41-4AF5-4975-BF91-3AC5F0B8D66B}"/>
+    <workbookView xWindow="30150" yWindow="2250" windowWidth="25200" windowHeight="11700" xr2:uid="{08943A41-4AF5-4975-BF91-3AC5F0B8D66B}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="44">
   <si>
     <t>manufacturer</t>
   </si>
@@ -162,6 +162,12 @@
   </si>
   <si>
     <t>GRM155C80J106ME11D</t>
+  </si>
+  <si>
+    <t>x7r</t>
+  </si>
+  <si>
+    <t>GRM21BZ71E106KE15L</t>
   </si>
 </sst>
 </file>
@@ -226,9 +232,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -266,7 +272,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -372,7 +378,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -514,7 +520,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -522,7 +528,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EEDD7F4B-E76F-430E-917C-19F8E46A1510}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
@@ -533,11 +539,11 @@
     <col min="6" max="7" width="22.85546875" customWidth="1"/>
     <col min="8" max="8" width="22.42578125" customWidth="1"/>
     <col min="9" max="9" width="23.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" customWidth="1"/>
+    <col min="11" max="11" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
@@ -568,8 +574,11 @@
       <c r="J1" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -600,8 +609,11 @@
       <c r="J2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -632,8 +644,11 @@
       <c r="J3">
         <v>402</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -656,7 +671,7 @@
         <v>100</v>
       </c>
       <c r="H4">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="I4">
         <v>16</v>
@@ -664,8 +679,11 @@
       <c r="J4">
         <v>6.3</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -697,8 +715,11 @@
       <c r="J5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K5">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
@@ -729,8 +750,11 @@
       <c r="J6">
         <v>1.4</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>34</v>
       </c>
@@ -753,7 +777,7 @@
         <v>21</v>
       </c>
       <c r="H7">
-        <v>8</v>
+        <v>12.5</v>
       </c>
       <c r="I7">
         <v>3.4</v>
@@ -761,8 +785,11 @@
       <c r="J7">
         <v>2.2000000000000002</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K7">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -785,7 +812,7 @@
         <v>60</v>
       </c>
       <c r="H8">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I8">
         <v>9.1999999999999993</v>
@@ -793,8 +820,11 @@
       <c r="J8">
         <v>6.1</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -817,7 +847,7 @@
         <v>2E-3</v>
       </c>
       <c r="H9">
-        <v>1.5E-3</v>
+        <v>2E-3</v>
       </c>
       <c r="I9">
         <v>4.0000000000000001E-3</v>
@@ -825,8 +855,11 @@
       <c r="J9">
         <v>5.0000000000000001E-3</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9">
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -858,8 +891,11 @@
       <c r="J10">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -890,8 +926,11 @@
       <c r="J11" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -921,6 +960,9 @@
       </c>
       <c r="J12">
         <v>20</v>
+      </c>
+      <c r="K12">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>